<commit_message>
changed output to outputs directory
</commit_message>
<xml_diff>
--- a/outputs/AAPL_analysis.xlsx
+++ b/outputs/AAPL_analysis.xlsx
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.005434875405307009</v>
+        <v>-0.005386687796610265</v>
       </c>
     </row>
     <row r="6">
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>-0.6866078203571274</v>
+        <v>-0.6879849593888123</v>
       </c>
     </row>
     <row r="5">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>251.49</v>
+        <v>252.6</v>
       </c>
     </row>
     <row r="6">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>-0.005434875405307009</v>
+        <v>-0.005386687796610265</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Multi-stage DCF + ROIC-based growth upgrade; removed heuristics, added CAPM discounting and projection-level transparency.
</commit_message>
<xml_diff>
--- a/outputs/AAPL_analysis.xlsx
+++ b/outputs/AAPL_analysis.xlsx
@@ -11,8 +11,7 @@
     <sheet name="02_Events" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="03_Risk" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="04_Data_Inputs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="05_Event_Impact" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="06_Valuation_Signal" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="05_Valuation_Model" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1725,7 +1724,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.03</v>
+        <v>0.04169402661947702</v>
       </c>
     </row>
     <row r="3">
@@ -1735,7 +1734,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.10338</v>
+        <v>0.10288</v>
       </c>
     </row>
     <row r="4">
@@ -1745,7 +1744,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04389999999999999</v>
+        <v>0.0434</v>
       </c>
     </row>
     <row r="5">
@@ -1755,7 +1754,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.005386687796610265</v>
+        <v>-0.004805317305218909</v>
       </c>
     </row>
     <row r="6">
@@ -1789,243 +1788,463 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Total Growth Adjustment</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Total Discount Adjustment</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.001842105263157896</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Event Count</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
+          <t>--- SIGNAL &amp; VALUATION ---</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Signal</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Bearish</t>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Confidence Level</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Strong Bearish</t>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Bearish</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Upside (%)</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>-0.6879849593888123</v>
+          <t>Confidence Level</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Strong Bearish</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Market Price</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>252.6</v>
+          <t>Upside (%)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>-0.700413561885859</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Shares Outstanding</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>14681140000</v>
+          <t>Market Price</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>251.64</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Intrinsic Value (Total)</t>
+          <t>Shares Outstanding</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1157094038212.261</v>
+        <v>14681140000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Intrinsic Value (Per Share)</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>78.81499925838602</v>
+          <t>Intrinsic Value (Total)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1106780773535.45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5Y PV Cash Flows</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>273687007491.1263</v>
+          <t>Intrinsic Value (Per Share)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>75.38793128704243</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Terminal Value</t>
+          <t>5Y PV Cash Flows</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1328340891894.227</v>
+        <v>277766565958.5085</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Terminal Value Contribution (%)</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>0.7634703849014904</v>
+          <t>Terminal Value</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1265250211041.656</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Growth Used</t>
+          <t>Terminal Value Contribution (%)</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.055</v>
+        <v>0.7490319920617851</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Discount Used</t>
+          <t>Stage 1 Growth</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.06923506654869256</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Raw ERP</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>-0.005386687796610265</v>
+          <t>Discount Used</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>0.08823549947915339</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Adjusted ERP</t>
+          <t>Raw ERP</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>0.03</v>
+        <v>-0.004805317305218909</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Driver 1</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>ERP floor applied (conservative risk adjustment)</t>
-        </is>
+          <t>Adjusted ERP</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>0.03</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Driver 1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Tight discount-growth spread (valuation sensitive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Driver 2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ERP floor applied (conservative risk adjustment)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Driver 3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Market pricing implies overvaluation</t>
         </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>--- EVENT IMPACT ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Total Growth Adjustment</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Total Discount Adjustment</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>0.01135549947915339</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Event Count</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>--- DIAGNOSTICS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Base CF</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>59494200000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Final Year CF</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>78057296645.19353</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Stage 1 Growth</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>0.06923506654869256</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Terminal Growth</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Discount Rate</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>0.08823549947915339</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Spread (Discount - Growth)</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>0.01900043293046083</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Terminal Value Contribution (%)</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>0.7490319920617851</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ROIC</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Reinvestment Rate</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>--- PROJECTION DETAILS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>growth</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>projected_cf</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>discounted_cf</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>0.06923506654869256</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>63613284896.26122</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>58455439954.59396</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>0.06923506654869256</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>68017554909.43481</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>57434816507.91405</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B43" s="4" t="n">
+        <v>0.06923506654869256</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>72726754850.06888</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>56432012997.5946</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>0.04711753327434628</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>76153460141.65222</v>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>54299781872.60841</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>5</v>
+      </c>
+      <c r="B45" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C45" t="n">
+        <v>78057296645.19353</v>
+      </c>
+      <c r="D45" t="n">
+        <v>51144514625.79752</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upgrade DCF Engine with Equity Valuation and Scenario Analysis
</commit_message>
<xml_diff>
--- a/outputs/AAPL_analysis.xlsx
+++ b/outputs/AAPL_analysis.xlsx
@@ -12,6 +12,7 @@
     <sheet name="03_Risk" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="04_Data_Inputs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="05_Valuation_Model" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="07_Scenario_Analysis" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,233 +588,253 @@
         <v>59494200000</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cash &amp; Equivalents</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-175000000</v>
+      </c>
+    </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>--- MARGINS ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+          <t>Total Debt</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>100327000000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>QoQ Delta</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>0.03016189390527432</v>
+          <t>--- MARGINS ---</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>YoY Delta</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>-0.0006640158925291795</v>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Trend Direction</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Compression</t>
-        </is>
+          <t>QoQ Delta</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.03016189390527432</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Primary Driver</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
+          <t>YoY Delta</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>-0.0006640158925291795</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Structural Assessment</t>
+          <t>Trend Direction</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Temporary Movement</t>
+          <t>Compression</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Risk Persistence Score</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>0.5</v>
+          <t>Primary Driver</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Structural Assessment</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Temporary Movement</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>--- WORKING CAPITAL ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+          <t>Risk Persistence Score</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pattern Classification</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Credit Deterioration</t>
+          <t>--- WORKING CAPITAL ---</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Working Capital Direction</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Deteriorating</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cash Efficiency Signal</t>
+          <t>Pattern Classification</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Cash Headwind</t>
+          <t>Credit Deterioration</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Operational Stress Flag</t>
-        </is>
-      </c>
-      <c r="B31" t="b">
-        <v>1</v>
+          <t>Working Capital Direction</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Deteriorating</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DSO_YoY</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>49.02803373943992</v>
+          <t>Cash Efficiency Signal</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Cash Headwind</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DIO_YoY</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>-21.54883431768032</v>
+          <t>Operational Stress Flag</t>
+        </is>
+      </c>
+      <c r="B33" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DPO_YoY</t>
+          <t>DSO_YoY</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>-11.41305323888341</v>
+        <v>49.02803373943992</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CCC_YoY</t>
+          <t>DIO_YoY</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>38.892252660643</v>
+        <v>-21.54883431768032</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DSO_QoQ</t>
+          <t>DPO_YoY</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>102.6812605233993</v>
+        <v>-11.41305323888341</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DIO_QoQ</t>
+          <t>CCC_YoY</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>38.892252660643</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DPO_QoQ</t>
+          <t>DSO_QoQ</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0</v>
+        <v>102.6812605233993</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>DIO_QoQ</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DPO_QoQ</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>CCC_QoQ</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B41" t="n">
         <v>102.6812605233993</v>
       </c>
     </row>
@@ -1754,7 +1775,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.004805317305218909</v>
+        <v>-0.00498059727956051</v>
       </c>
     </row>
     <row r="6">
@@ -1788,7 +1809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1841,7 +1862,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>-0.700413561885859</v>
+        <v>-0.7283302512419871</v>
       </c>
     </row>
     <row r="6">
@@ -1851,7 +1872,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>251.64</v>
+        <v>252.3</v>
       </c>
     </row>
     <row r="7">
@@ -1867,7 +1888,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Intrinsic Value (Total)</t>
+          <t>Enterprise Value</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -1877,374 +1898,502 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Intrinsic Value (Per Share)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>75.38793128704243</v>
+          <t>Net Debt</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>100502000000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5Y PV Cash Flows</t>
+          <t>Equity Value</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>277766565958.5085</v>
+        <v>1006278773535.45</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Terminal Value</t>
+          <t>Intrinsic Value (Total)</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1265250211041.656</v>
+        <v>1006278773535.45</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Terminal Value Contribution (%)</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>0.7490319920617851</v>
+          <t>Intrinsic Value (Per Share)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>68.54227761164665</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Stage 1 Growth</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>0.06923506654869256</v>
+          <t>5Y PV Cash Flows</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>277766565958.5085</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Discount Used</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>0.08823549947915339</v>
+          <t>Terminal Value</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1265250211041.656</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Raw ERP</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>-0.004805317305218909</v>
+          <t>Terminal Value Contribution (%)</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>0.7490319920617851</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Adjusted ERP</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>0.03</v>
+          <t>Stage 1 Growth</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>0.06923506654869256</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Driver 1</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Tight discount-growth spread (valuation sensitive)</t>
-        </is>
+          <t>Discount Used</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>0.08823549947915339</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Driver 2</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>ERP floor applied (conservative risk adjustment)</t>
-        </is>
+          <t>Raw ERP</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>-0.00498059727956051</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Driver 3</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Market pricing implies overvaluation</t>
+          <t>Adjusted ERP</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Driver 1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Tight discount-growth spread (valuation sensitive)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>--- EVENT IMPACT ---</t>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Driver 2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ERP floor applied (conservative risk adjustment)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Driver 3</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Total Growth Adjustment</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>0</v>
+          <t>Market pricing implies overvaluation</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Total Discount Adjustment</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>0.01135549947915339</v>
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>--- EVENT IMPACT ---</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Event Count</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>38</v>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Total Growth Adjustment</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>--- DIAGNOSTICS ---</t>
-        </is>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Total Discount Adjustment</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>0.01135549947915339</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Base CF</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>59494200000</v>
+          <t>Event Count</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Final Year CF</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>78057296645.19353</v>
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>--- DIAGNOSTICS ---</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Stage 1 Growth</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n">
-        <v>0.06923506654869256</v>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Terminal Growth</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="n">
-        <v>0.025</v>
+          <t>Base CF</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>59494200000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Discount Rate</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="n">
-        <v>0.08823549947915339</v>
+          <t>Final Year CF</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>78057296645.19353</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Spread (Discount - Growth)</t>
+          <t>Stage 1 Growth</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>0.01900043293046083</v>
+        <v>0.06923506654869256</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Terminal Value Contribution (%)</t>
+          <t>Terminal Growth</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
-        <v>0.7490319920617851</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ROIC</t>
+          <t>Discount Rate</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>0.5</v>
+        <v>0.08823549947915339</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Reinvestment Rate</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>0.1</v>
+          <t>Spread (Discount - Growth)</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>0.01900043293046083</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Terminal Value Contribution (%)</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>0.7490319920617851</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="inlineStr">
-        <is>
-          <t>--- PROJECTION DETAILS ---</t>
-        </is>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ROIC</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>Reinvestment Rate</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>--- PROJECTION DETAILS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>growth</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>projected_cf</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>discounted_cf</t>
         </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B41" s="4" t="n">
-        <v>0.06923506654869256</v>
-      </c>
-      <c r="C41" s="5" t="n">
-        <v>63613284896.26122</v>
-      </c>
-      <c r="D41" s="5" t="n">
-        <v>58455439954.59396</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B42" s="4" t="n">
-        <v>0.06923506654869256</v>
-      </c>
-      <c r="C42" s="5" t="n">
-        <v>68017554909.43481</v>
-      </c>
-      <c r="D42" s="5" t="n">
-        <v>57434816507.91405</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B43" s="4" t="n">
-        <v>0.06923506654869256</v>
-      </c>
-      <c r="C43" s="5" t="n">
-        <v>72726754850.06888</v>
-      </c>
-      <c r="D43" s="5" t="n">
-        <v>56432012997.5946</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>0.06923506654869256</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>63613284896.26122</v>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>58455439954.59396</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="4" t="n">
+        <v>0.06923506654869256</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>68017554909.43481</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>57434816507.91405</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>0.06923506654869256</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>72726754850.06888</v>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>56432012997.5946</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B44" s="4" t="n">
+      <c r="B47" s="4" t="n">
         <v>0.04711753327434628</v>
       </c>
-      <c r="C44" s="5" t="n">
+      <c r="C47" s="5" t="n">
         <v>76153460141.65222</v>
       </c>
-      <c r="D44" s="5" t="n">
+      <c r="D47" s="5" t="n">
         <v>54299781872.60841</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="n">
+    <row r="48">
+      <c r="A48" t="n">
         <v>5</v>
       </c>
-      <c r="B45" t="n">
+      <c r="B48" t="n">
         <v>0.025</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C48" t="n">
         <v>78057296645.19353</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D48" t="n">
         <v>51144514625.79752</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Intrinsic Value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Upside</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>736669053995.5182</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>-0.8011180379830252</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>0.05538805323895405</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>0.1049754994791534</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>1006278773535.45</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>-0.7283302512419871</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>0.06923506654869256</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>0.08823549947915339</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>831810025739.7334</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>-0.7754323884690899</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.08308207985843107</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.1030820798584311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Sensitivity Analysis matrix to DCF engine
</commit_message>
<xml_diff>
--- a/outputs/AAPL_analysis.xlsx
+++ b/outputs/AAPL_analysis.xlsx
@@ -13,6 +13,7 @@
     <sheet name="04_Data_Inputs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="05_Valuation_Model" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="07_Scenario_Analysis" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="08_Sensitivity_Analysis" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -60,7 +63,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -68,6 +71,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1755,7 +1759,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.10288</v>
+        <v>0.10338</v>
       </c>
     </row>
     <row r="4">
@@ -1765,7 +1769,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0434</v>
+        <v>0.04389999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -1775,7 +1779,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.00498059727956051</v>
+        <v>-0.005519204399114672</v>
       </c>
     </row>
     <row r="6">
@@ -1862,7 +1866,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>-0.7283302512419871</v>
+        <v>-0.7310376619187224</v>
       </c>
     </row>
     <row r="6">
@@ -1872,7 +1876,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>252.3</v>
+        <v>252.62</v>
       </c>
     </row>
     <row r="7">
@@ -1892,7 +1896,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1106780773535.45</v>
+        <v>1098015960223.7</v>
       </c>
     </row>
     <row r="9">
@@ -1912,7 +1916,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1006278773535.45</v>
+        <v>997513960223.7003</v>
       </c>
     </row>
     <row r="11">
@@ -1922,7 +1926,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1006278773535.45</v>
+        <v>997513960223.7003</v>
       </c>
     </row>
     <row r="12">
@@ -1932,7 +1936,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>68.54227761164665</v>
+        <v>67.94526584609235</v>
       </c>
     </row>
     <row r="13">
@@ -1942,7 +1946,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>277766565958.5085</v>
+        <v>277392253579.6608</v>
       </c>
     </row>
     <row r="14">
@@ -1952,7 +1956,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1265250211041.656</v>
+        <v>1255324422263.179</v>
       </c>
     </row>
     <row r="15">
@@ -1962,7 +1966,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.7490319920617851</v>
+        <v>0.7473695614377525</v>
       </c>
     </row>
     <row r="16">
@@ -1982,7 +1986,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.08823549947915339</v>
+        <v>0.08873549947915339</v>
       </c>
     </row>
     <row r="18">
@@ -1992,7 +1996,7 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>-0.00498059727956051</v>
+        <v>-0.005519204399114672</v>
       </c>
     </row>
     <row r="19">
@@ -2156,7 +2160,7 @@
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>0.08823549947915339</v>
+        <v>0.08873549947915339</v>
       </c>
     </row>
     <row r="37">
@@ -2166,7 +2170,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>0.01900043293046083</v>
+        <v>0.01950043293046083</v>
       </c>
     </row>
     <row r="38">
@@ -2176,7 +2180,7 @@
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>0.7490319920617851</v>
+        <v>0.7473695614377525</v>
       </c>
     </row>
     <row r="39">
@@ -2239,7 +2243,7 @@
         <v>63613284896.26122</v>
       </c>
       <c r="D44" s="5" t="n">
-        <v>58455439954.59396</v>
+        <v>58428594389.26494</v>
       </c>
     </row>
     <row r="45">
@@ -2253,7 +2257,7 @@
         <v>68017554909.43481</v>
       </c>
       <c r="D45" s="5" t="n">
-        <v>57434816507.91405</v>
+        <v>57382074930.0813</v>
       </c>
     </row>
     <row r="46">
@@ -2267,7 +2271,7 @@
         <v>72726754850.06888</v>
       </c>
       <c r="D46" s="5" t="n">
-        <v>56432012997.5946</v>
+        <v>56354299768.78634</v>
       </c>
     </row>
     <row r="47">
@@ -2281,7 +2285,7 @@
         <v>76153460141.65222</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>54299781872.60841</v>
+        <v>54200102220.90173</v>
       </c>
     </row>
     <row r="48">
@@ -2295,7 +2299,7 @@
         <v>78057296645.19353</v>
       </c>
       <c r="D48" t="n">
-        <v>51144514625.79752</v>
+        <v>51027182270.62644</v>
       </c>
     </row>
   </sheetData>
@@ -2346,16 +2350,16 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>736669053995.5182</v>
+        <v>731426136853.2622</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>-0.8011180379830252</v>
+        <v>-0.80278362835374</v>
       </c>
       <c r="D2" s="6" t="n">
         <v>0.05538805323895405</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>0.1049754994791534</v>
+        <v>0.1054754994791534</v>
       </c>
     </row>
     <row r="3">
@@ -2365,16 +2369,16 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>1006278773535.45</v>
+        <v>997513960223.7003</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>-0.7283302512419871</v>
+        <v>-0.7310376619187224</v>
       </c>
       <c r="D3" s="6" t="n">
         <v>0.06923506654869256</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>0.08823549947915339</v>
+        <v>0.08873549947915339</v>
       </c>
     </row>
     <row r="4">
@@ -2387,13 +2391,248 @@
         <v>831810025739.7334</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>-0.7754323884690899</v>
+        <v>-0.7757168538150241</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>0.08308207985843107</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>0.1030820798584311</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Growth Rate</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>7.0%</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>8.0%</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>9.0%</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>86.96131101218172</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>69.89140126856249</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>58.07410742217829</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>49.40837190210377</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>42.78187058802786</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>37.55062675921888</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>90.01959173501793</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>72.36457204970058</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>60.14289634050361</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>51.18119259875603</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>44.32885357653025</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>38.91973946915284</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>93.15185958279734</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>74.89710832657362</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>62.26095835416056</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>52.99591046496124</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>45.9121146367611</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>40.32071243537611</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>96.35928227418276</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>77.48994272066746</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>64.42906397208012</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>54.85317766387584</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>47.53221588570802</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>41.75403707455268</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>66.6479894802048</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>80.14401487225619</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>66.6479894802048</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>56.75365123008976</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>49.18972362355476</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>43.22020844684365</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>0.08000000000000002</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>58.69799306962638</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>58.69799306962638</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>68.91851694148886</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>58.69799306962639</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>50.88520833368126</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>44.7197252559071</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>0.09000000000000001</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>52.61924468266356</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>52.61924468266356</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>52.61924468266356</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>60.68686995994259</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>52.61924468266363</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>46.25308984889815</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>47.82080821646895</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>47.82080821646895</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>47.82080821646895</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>47.82080821646895</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>54.39241152027419</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>47.82080821646901</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement Investment Memo Output Layer
</commit_message>
<xml_diff>
--- a/outputs/AAPL_analysis.xlsx
+++ b/outputs/AAPL_analysis.xlsx
@@ -14,6 +14,7 @@
     <sheet name="05_Valuation_Model" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="07_Scenario_Analysis" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="08_Sensitivity_Analysis" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="09_Investment_Memo" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -63,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -72,6 +73,9 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2638,4 +2642,279 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>The model estimates an intrinsic value of $67.95, implying -73.1% upside from the current price of $252.62.
+Under a bear case, value falls to $49.82, while the bull case reaches $56.66.
+Growth is driven by an estimated ROIC of 50.0% and reinvestment rate of 10.0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>--- SUMMARY ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Investment Signal</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Intrinsic Value (Base Case)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>67.94526584609235</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Current Price</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>252.62</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Upside (%)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>-0.7310376619187224</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>--- SCENARIOS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Bear Value</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>49.82079980527821</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Base Value</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>67.94526584609235</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Bull Value</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>56.65840838924861</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>--- DRIVERS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Growth Assumption (Stage 1)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>0.06923506654869256</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Discount Rate</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>0.08873549947915339</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ROIC</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Reinvestment Rate</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>--- RISK SUMMARY ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Key Risks</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Debt issuance announced, Debt issuance announced, Executive leadership change, CEO leadership change, Debt issuance announced, Debt issuance announced, CEO leadership change, CEO leadership change, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, CFO leadership change, Debt issuance announced, Debt issuance announced, CEO leadership change, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Risk Score</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>--- VALUATION DIAGNOSTICS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Terminal Value Contribution (%)</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>0.7473695614377525</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Spread (Discount - Growth)</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.01950043293046083</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Integrate Gemini 2.5 Generative AI for native SEC 8-K event extraction
</commit_message>
<xml_diff>
--- a/outputs/AAPL_analysis.xlsx
+++ b/outputs/AAPL_analysis.xlsx
@@ -857,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -868,17 +868,42 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Event Category</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Event Type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Event Summary</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Event Risk Score</t>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Structured Context</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Financial Interpretation</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Time Decay Factor</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Adjusted Risk Score</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Event Weight</t>
         </is>
       </c>
     </row>
@@ -890,756 +915,242 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Debt Issuance</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>70</v>
+          <t>Annual Shareholder Meeting Outcomes</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Apple Inc. shareholders, at their Annual Meeting on February 24, 2026, re-elected all directors, ratified Ernst &amp; Young LLP as the independent auditor, approved executive compensation, and approved an amended Non-Employee Director Stock Plan, while rejecting a shareholder proposal for a 'China Entanglement Audit'.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{'Meeting Date': 'February 24, 2026', 'Company': 'Apple Inc.', 'Directors Re-elected': 'Wanda Austin, Tim Cook, Alex Gorsky, Andrea Jung, Art Levinson, Monica Lozano, Ron Sugar, Sue Wagner', 'Auditor Ratification Status': 'Approved (Ernst &amp; Young LLP for fiscal year 2026)', 'Executive Compensation Approval Status': 'Approved', 'Non-Employee Director Stock Plan Approval Status': 'Approved (Apple Inc. Non-Employee Director Stock Plan, as Amended and Restated)', 'Shareholder Proposal (China Entanglement Audit) Status': 'Not Approved'}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>{'Board Stability': 'Maintained, with all incumbent directors re-elected.', 'Corporate Oversight': 'Continued by existing board and independent auditor.', 'Executive Incentives': 'Shareholder endorsement of current executive compensation practices.', 'Equity Compensation': 'Potential for future share dilution due to the approval of the Non-Employee Director Stock Plan.', 'Strategic Direction': "Shareholders supported management's existing strategy by rejecting the China Entanglement Audit proposal."}</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0.961</v>
+      </c>
+      <c r="H2" t="n">
+        <v>50</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.481</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Debt Issuance</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>70</v>
+          <t>Non-Employee Director Stock Plan Amendment</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Apple Inc. amended and restated its Non-Employee Director Stock Plan, effective February 24, 2026, to update the framework for granting equity awards, including Restricted Stock Units and Options, to its non-employee directors.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{'Plan Name': 'Apple Inc. Non-Employee Director Stock Plan', 'Effective Date': 'February 24, 2026', 'Board Adoption Date': 'November 4, 2025', 'Maximum Shares for Awards': '44,800,000 Shares', 'RSU Annual Grant Value': '$310,000', 'Annual Compensation Limit for Non-Employee Directors': '$1,500,000', 'Plan Termination Date': 'February 23, 2036'}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>{'Potential Dilution': "Potential for increased share dilution up to 44,800,000 shares over the plan's life, as RSUs count as two shares for every one issued, which could impact earnings per share.", 'Compensation Structure': 'Establishes a standardized framework for non-employee director equity compensation, aiming to align incentives with long-term shareholder value and impacting future compensation expenses.', 'Governance Impact': "Strengthens director retention and motivation by directly tying a significant portion of non-employee director compensation to the company's stock performance."}</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.961</v>
+      </c>
+      <c r="H3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.481</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Governance Change</t>
+          <t>Capital Structure</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Executive leadership change</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>60</v>
+          <t>Dividend Declaration</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Apple's board of directors declared a cash dividend of $0.26 per share of common stock, payable on February 12, 2026, to shareholders of record as of February 9, 2026.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{'Dividend Per Share': '$0.26', 'Record Date': 'February 9, 2026', 'Payment Date': 'February 12, 2026'}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>{'Shareholder Returns': 'Consistent', 'Cash Outflow': 'Projected Increase', 'Equity': 'Projected Decrease'}</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="H4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.464</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2024-05-03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Governance Change</t>
+          <t>Legal / Regulatory</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CEO leadership change</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>60</v>
+          <t>Preliminary Settlement Approval for Shareholder Derivative Lawsuits</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>A U.S. District Court granted preliminary approval for the proposed settlement of consolidated shareholder derivative lawsuits against Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{'Date of Order': 'April 23, 2024', 'Court': 'U.S. District Court for the Northern District of California', 'Primary Case Name': 'In re Apple Inc. Stockholder Derivative Litigation', 'Primary Case Number': '4:19-cv-05153-YGR (N.D. Cal.)', 'Related Case Number': '19CV355213 (Cal. Super. Ct., Santa Clara County)'}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>{'Litigation Risk': 'Decreased', 'Uncertainty': 'Reduced regarding litigation outcome', 'Future Cash Outflow': 'Possible, pending final settlement terms and approval', 'Legal Expenses': 'Anticipated to decrease as settlement progresses'}</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="H5" t="n">
+        <v>80</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.311</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-10-30</t>
+          <t>2024-08-23</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Debt Issuance</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>70</v>
+          <t>Bylaws Amendment</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Apple Inc.'s Board of Directors approved and adopted amended and restated bylaws, effective August 20, 2024, to revise procedural mechanics and disclosure requirements for shareholder nominations of directors and submission of other proposals at shareholder meetings.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{'Company': 'Apple Inc.', 'Effective Date': 'August 20, 2024'}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>{'Shareholder Influence': 'Potentially Reduced', 'Board Autonomy': 'Potentially Enhanced', 'Governance Clarity': 'Improved'}</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="H6" t="n">
+        <v>50</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.226</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-07-31</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Debt Issuance</t>
+          <t>Capital Structure</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2025-07-25</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Governance Change</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CEO leadership change</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2025-07-09</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Governance Change</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CEO leadership change</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2025-05-12</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2025-05-01</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2025-02-25</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2025-01-30</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2025-01-03</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Governance Change</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>CFO leadership change</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2024-10-31</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2024-09-10</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2024-08-26</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Governance Change</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CEO leadership change</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2024-08-23</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2024-08-01</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2024-05-03</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2024-05-02</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2024-02-28</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2024-02-01</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2023-11-02</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2023-08-03</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2023-05-10</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2023-05-04</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2023-03-10</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2023-02-02</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2022-10-27</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2022-07-28</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2022-04-28</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2022-01-27</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2021-10-28</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2021-07-27</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2021-04-28</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2021-01-27</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2020-10-29</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2020-07-30</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Debt Issuance</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Debt issuance announced</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>70</v>
+          <t>Cash Dividend Declaration</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Apple Inc.'s board of directors declared a cash dividend of $0.25 per share of the Company's common stock.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{'Dividend Per Share': '$0.25', 'Record Date': 'August 12, 2024', 'Payment Date': 'August 15, 2024'}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>{'Shareholder Returns': 'Direct return of capital to shareholders', 'Cash Flow Impact': 'Future cash outflow for dividend payment', 'Capital Allocation Strategy': 'Demonstrates an ongoing commitment to shareholder distributions'}</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0.439</v>
+      </c>
+      <c r="H7" t="n">
+        <v>50</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.22</v>
       </c>
     </row>
   </sheetData>
@@ -1870,7 +1381,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>-0.7310376619187224</v>
+        <v>-0.6662322494870978</v>
       </c>
     </row>
     <row r="6">
@@ -1900,7 +1411,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1098015960223.7</v>
+        <v>1338363006801.892</v>
       </c>
     </row>
     <row r="9">
@@ -1920,7 +1431,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>997513960223.7003</v>
+        <v>1237861006801.892</v>
       </c>
     </row>
     <row r="11">
@@ -1930,7 +1441,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>997513960223.7003</v>
+        <v>1237861006801.892</v>
       </c>
     </row>
     <row r="12">
@@ -1940,7 +1451,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>67.94526584609235</v>
+        <v>84.31640913456937</v>
       </c>
     </row>
     <row r="13">
@@ -1950,7 +1461,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>277392253579.6608</v>
+        <v>286092661542.4216</v>
       </c>
     </row>
     <row r="14">
@@ -1960,7 +1471,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1255324422263.179</v>
+        <v>1527467145118.812</v>
       </c>
     </row>
     <row r="15">
@@ -1970,7 +1481,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.7473695614377525</v>
+        <v>0.7862368728899202</v>
       </c>
     </row>
     <row r="16">
@@ -1990,7 +1501,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.08873549947915339</v>
+        <v>0.07738</v>
       </c>
     </row>
     <row r="18">
@@ -2085,7 +1596,7 @@
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>0.01135549947915339</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -2095,7 +1606,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -2164,7 +1675,7 @@
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>0.08873549947915339</v>
+        <v>0.07738</v>
       </c>
     </row>
     <row r="37">
@@ -2174,7 +1685,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>0.01950043293046083</v>
+        <v>0.008144933451307443</v>
       </c>
     </row>
     <row r="38">
@@ -2184,7 +1695,7 @@
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>0.7473695614377525</v>
+        <v>0.7862368728899202</v>
       </c>
     </row>
     <row r="39">
@@ -2247,7 +1758,7 @@
         <v>63613284896.26122</v>
       </c>
       <c r="D44" s="5" t="n">
-        <v>58428594389.26494</v>
+        <v>59044427125.30511</v>
       </c>
     </row>
     <row r="45">
@@ -2261,7 +1772,7 @@
         <v>68017554909.43481</v>
       </c>
       <c r="D45" s="5" t="n">
-        <v>57382074930.0813</v>
+        <v>58598054508.76667</v>
       </c>
     </row>
     <row r="46">
@@ -2275,7 +1786,7 @@
         <v>72726754850.06888</v>
       </c>
       <c r="D46" s="5" t="n">
-        <v>56354299768.78634</v>
+        <v>58155056444.62032</v>
       </c>
     </row>
     <row r="47">
@@ -2289,7 +1800,7 @@
         <v>76153460141.65222</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>54200102220.90173</v>
+        <v>56521542307.93333</v>
       </c>
     </row>
     <row r="48">
@@ -2303,7 +1814,7 @@
         <v>78057296645.19353</v>
       </c>
       <c r="D48" t="n">
-        <v>51027182270.62644</v>
+        <v>53773581155.79616</v>
       </c>
     </row>
   </sheetData>
@@ -2354,16 +1865,16 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>731426136853.2622</v>
+        <v>869215489659.3091</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>-0.80278362835374</v>
+        <v>-0.7656311192448856</v>
       </c>
       <c r="D2" s="6" t="n">
         <v>0.05538805323895405</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>0.1054754994791534</v>
+        <v>0.09412</v>
       </c>
     </row>
     <row r="3">
@@ -2373,16 +1884,16 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>997513960223.7003</v>
+        <v>1237861006801.892</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>-0.7310376619187224</v>
+        <v>-0.6662322494870978</v>
       </c>
       <c r="D3" s="6" t="n">
         <v>0.06923506654869256</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>0.08873549947915339</v>
+        <v>0.07738</v>
       </c>
     </row>
     <row r="4">
@@ -2659,8 +2170,8 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>The model estimates an intrinsic value of $67.95, implying -73.1% upside from the current price of $252.62.
-Under a bear case, value falls to $49.82, while the bull case reaches $56.66.
+          <t>The model estimates an intrinsic value of $84.32, implying -66.6% upside from the current price of $252.62.
+Under a bear case, value falls to $59.21, while the bull case reaches $56.66.
 Growth is driven by an estimated ROIC of 50.0% and reinvestment rate of 10.0%.</t>
         </is>
       </c>
@@ -2703,7 +2214,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>67.94526584609235</v>
+        <v>84.31640913456937</v>
       </c>
     </row>
     <row r="7">
@@ -2723,7 +2234,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.7310376619187224</v>
+        <v>-0.6662322494870978</v>
       </c>
     </row>
     <row r="10">
@@ -2752,7 +2263,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>49.82079980527821</v>
+        <v>59.206266656357</v>
       </c>
     </row>
     <row r="13">
@@ -2762,7 +2273,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>67.94526584609235</v>
+        <v>84.31640913456937</v>
       </c>
     </row>
     <row r="14">
@@ -2811,7 +2322,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>0.08873549947915339</v>
+        <v>0.07738</v>
       </c>
     </row>
     <row r="20">
@@ -2861,7 +2372,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Debt issuance announced, Debt issuance announced, Executive leadership change, CEO leadership change, Debt issuance announced, Debt issuance announced, CEO leadership change, CEO leadership change, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, CFO leadership change, Debt issuance announced, Debt issuance announced, CEO leadership change, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced, Debt issuance announced</t>
+          <t>A U.S. District Court granted preliminary approval for the proposed settlement of consolidated shareholder derivative lawsuits against Apple Inc.</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2412,7 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>0.7473695614377525</v>
+        <v>0.7862368728899202</v>
       </c>
     </row>
     <row r="31">
@@ -2911,7 +2422,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.01950043293046083</v>
+        <v>0.008144933451307443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement Revenue-to-FCF pipeline and unified Investment Decision Layer
</commit_message>
<xml_diff>
--- a/outputs/AAPL_analysis.xlsx
+++ b/outputs/AAPL_analysis.xlsx
@@ -73,7 +73,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -920,32 +920,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Annual Shareholder Meeting Outcomes</t>
+          <t>Non-Employee Director Equity Plan Amendment</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Apple Inc. shareholders, at their Annual Meeting on February 24, 2026, re-elected all directors, ratified Ernst &amp; Young LLP as the independent auditor, approved executive compensation, and approved an amended Non-Employee Director Stock Plan, while rejecting a shareholder proposal for a 'China Entanglement Audit'.</t>
+          <t>Apple Inc. amended and restated its Non-Employee Director Stock Plan, effective February 24, 2026, establishing an aggregate limit of 44.8 million shares for awards and an annual compensation cap of $1.5 million per non-employee director.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>{'Meeting Date': 'February 24, 2026', 'Company': 'Apple Inc.', 'Directors Re-elected': 'Wanda Austin, Tim Cook, Alex Gorsky, Andrea Jung, Art Levinson, Monica Lozano, Ron Sugar, Sue Wagner', 'Auditor Ratification Status': 'Approved (Ernst &amp; Young LLP for fiscal year 2026)', 'Executive Compensation Approval Status': 'Approved', 'Non-Employee Director Stock Plan Approval Status': 'Approved (Apple Inc. Non-Employee Director Stock Plan, as Amended and Restated)', 'Shareholder Proposal (China Entanglement Audit) Status': 'Not Approved'}</t>
+          <t>{'Effective Date': 'February 24, 2026', 'Maximum Shares for Awards': '44,800,000 Shares', 'Annual Director Compensation Cap': '$1,500,000', 'Annual RSU Grant Value': '$310,000', 'Plan Expiration Date': 'February 23, 2036'}</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{'Board Stability': 'Maintained, with all incumbent directors re-elected.', 'Corporate Oversight': 'Continued by existing board and independent auditor.', 'Executive Incentives': 'Shareholder endorsement of current executive compensation practices.', 'Equity Compensation': 'Potential for future share dilution due to the approval of the Non-Employee Director Stock Plan.', 'Strategic Direction': "Shareholders supported management's existing strategy by rejecting the China Entanglement Audit proposal."}</t>
+          <t>{'Potential Share Dilution': 'Increase (due to additional shares authorized for issuance)', 'Compensation Expense': 'Ongoing (reflecting equity grants to directors)', 'Shareholder Alignment': 'Improved (incentivizes directors through stock ownership)'}</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.961</v>
+        <v>0.96</v>
       </c>
       <c r="H2" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="I2" t="n">
-        <v>0.481</v>
+        <v>0.576</v>
       </c>
     </row>
     <row r="3">
@@ -961,32 +961,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Non-Employee Director Stock Plan Amendment</t>
+          <t>Annual Shareholder Meeting Results</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Apple Inc. amended and restated its Non-Employee Director Stock Plan, effective February 24, 2026, to update the framework for granting equity awards, including Restricted Stock Units and Options, to its non-employee directors.</t>
+          <t>Apple Inc. held its 2026 Annual Meeting of Shareholders on February 24, 2026, where all nominated directors were elected, the appointment of Ernst &amp; Young LLP as independent auditor was ratified, an advisory resolution to approve executive compensation was approved, the Non-Employee Director Stock Plan, as Amended and Restated, was approved, and a shareholder proposal for a 'China Entanglement Audit' was not approved.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{'Plan Name': 'Apple Inc. Non-Employee Director Stock Plan', 'Effective Date': 'February 24, 2026', 'Board Adoption Date': 'November 4, 2025', 'Maximum Shares for Awards': '44,800,000 Shares', 'RSU Annual Grant Value': '$310,000', 'Annual Compensation Limit for Non-Employee Directors': '$1,500,000', 'Plan Termination Date': 'February 23, 2036'}</t>
+          <t>{'Meeting Date': 'February 24, 2026', 'Company': 'Apple Inc.', 'Directors Elected': 'Wanda Austin, Tim Cook, Alex Gorsky, Andrea Jung, Art Levinson, Monica Lozano, Ron Sugar, Sue Wagner', 'Auditor Ratified': 'Ernst &amp; Young LLP', 'Executive Compensation Approved': 'Yes', 'Non-Employee Director Stock Plan Approved': 'Yes', "Shareholder Proposal 'China Entanglement Audit' Approved": 'No'}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{'Potential Dilution': "Potential for increased share dilution up to 44,800,000 shares over the plan's life, as RSUs count as two shares for every one issued, which could impact earnings per share.", 'Compensation Structure': 'Establishes a standardized framework for non-employee director equity compensation, aiming to align incentives with long-term shareholder value and impacting future compensation expenses.', 'Governance Impact': "Strengthens director retention and motivation by directly tying a significant portion of non-employee director compensation to the company's stock performance."}</t>
+          <t>{'Board Continuity': 'Maintained', 'Executive Compensation Structure': 'Affirmed by shareholders', 'Director Compensation': 'Stock plan approved, allowing for continued equity-based incentives and related compensation expense', 'Operational Risk related to China': 'No immediate change in strategy as shareholder proposal for audit was rejected'}</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.961</v>
+        <v>0.96</v>
       </c>
       <c r="H3" t="n">
         <v>50</v>
       </c>
       <c r="I3" t="n">
-        <v>0.481</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="4">
@@ -1002,32 +1002,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Dividend Declaration</t>
+          <t>Shareholder Return Program</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Apple's board of directors declared a cash dividend of $0.26 per share of common stock, payable on February 12, 2026, to shareholders of record as of February 9, 2026.</t>
+          <t>Apple's board of directors declared a cash dividend of $0.26 per share, payable on February 12, 2026, and the company returned approximately $32 billion to shareholders during the first fiscal quarter through a combination of dividends and common stock repurchases.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>{'Dividend Per Share': '$0.26', 'Record Date': 'February 9, 2026', 'Payment Date': 'February 12, 2026'}</t>
+          <t>{'Total Shareholder Return Amount (Reported)': '$32 billion', 'Dividend Amount Per Share': '$0.26', 'Dividend Record Date': 'February 9, 2026', 'Dividend Payment Date': 'February 12, 2026', 'Common Stock Repurchases (Q1 2026)': '$24,701 million', 'Dividend Payments (Q1 2026)': '$3,921 million'}</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{'Shareholder Returns': 'Consistent', 'Cash Outflow': 'Projected Increase', 'Equity': 'Projected Decrease'}</t>
+          <t>{'Shareholder Value': 'Enhanced through direct returns of capital', 'Liquidity': 'Reduced due to significant cash outflow, but supported by strong operating cash flow', 'Equity Capital': 'Decreased as a result of repurchases and dividend payments', 'Earnings Per Share (EPS)': 'Accretive, due to the reduction in outstanding shares from repurchases', 'Capital Allocation': 'Reflects a continued aggressive return of capital strategy'}</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.927</v>
+        <v>0.926</v>
       </c>
       <c r="H4" t="n">
         <v>50</v>
       </c>
       <c r="I4" t="n">
-        <v>0.464</v>
+        <v>0.463</v>
       </c>
     </row>
     <row r="5">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Preliminary Settlement Approval for Shareholder Derivative Lawsuits</t>
+          <t>Lawsuit Settlement Approval</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>A U.S. District Court granted preliminary approval for the proposed settlement of consolidated shareholder derivative lawsuits against Apple Inc.</t>
+          <t>A U.S. District Court granted preliminary approval for the proposed settlement of consolidated shareholder derivative lawsuits against Apple Inc. on April 23, 2024.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>{'Date of Order': 'April 23, 2024', 'Court': 'U.S. District Court for the Northern District of California', 'Primary Case Name': 'In re Apple Inc. Stockholder Derivative Litigation', 'Primary Case Number': '4:19-cv-05153-YGR (N.D. Cal.)', 'Related Case Number': '19CV355213 (Cal. Super. Ct., Santa Clara County)'}</t>
+          <t>{'Date of Order': 'April 23, 2024', 'Court': 'U.S. District Court for the Northern District of California', 'Case Name': 'In re Apple Inc. Stockholder Derivative Litigation', 'Case Numbers': '4:19-cv-05153-YGR (N.D. Cal.) and 19CV355213 (Cal. Super. Ct., Santa Clara County)'}</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{'Litigation Risk': 'Decreased', 'Uncertainty': 'Reduced regarding litigation outcome', 'Future Cash Outflow': 'Possible, pending final settlement terms and approval', 'Legal Expenses': 'Anticipated to decrease as settlement progresses'}</t>
+          <t>{'Litigation Risk': 'Reduced', 'Legal Uncertainty': 'Decreased', 'Potential Cash Flow Impact': 'Implied Outflow (pending final settlement terms)', 'Reputational Impact': 'Potentially Mitigated'}</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -1068,54 +1068,54 @@
         <v>80</v>
       </c>
       <c r="I5" t="n">
-        <v>0.311</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-08-23</t>
+          <t>2024-05-02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Capital Structure</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bylaws Amendment</t>
+          <t>Share Repurchase Authorization &amp; Dividend Increase</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Apple Inc.'s Board of Directors approved and adopted amended and restated bylaws, effective August 20, 2024, to revise procedural mechanics and disclosure requirements for shareholder nominations of directors and submission of other proposals at shareholder meetings.</t>
+          <t>Apple's board of directors authorized an additional $110 billion for share repurchases and increased the quarterly cash dividend by 4 percent to $0.25 per share.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>{'Company': 'Apple Inc.', 'Effective Date': 'August 20, 2024'}</t>
+          <t>{'Share Repurchase Authorization Amount': '$110 billion', 'Quarterly Dividend per Share': '$0.25', 'Dividend Increase Percentage': '4%', 'Dividend Payable Date': 'May 16, 2024', 'Dividend Record Date': 'May 13, 2024'}</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{'Shareholder Influence': 'Potentially Reduced', 'Board Autonomy': 'Potentially Enhanced', 'Governance Clarity': 'Improved'}</t>
+          <t>{'Return to Shareholders': 'Increase', 'Share Count': 'Decrease (through repurchases)', 'EPS': 'Accretive (through repurchases)', 'Cash Outflow': 'Increase (for repurchases and dividends)'}</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.453</v>
+        <v>0.387</v>
       </c>
       <c r="H6" t="n">
         <v>50</v>
       </c>
       <c r="I6" t="n">
-        <v>0.226</v>
+        <v>0.194</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-08-01</t>
+          <t>2023-05-10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1125,32 +1125,32 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cash Dividend Declaration</t>
+          <t>Debt Issuance</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Apple Inc.'s board of directors declared a cash dividend of $0.25 per share of the Company's common stock.</t>
+          <t>Apple Inc. consummated the issuance and sale of $5.25 billion in aggregate principal amount across five series of senior unsecured notes with varying interest rates and maturities.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>{'Dividend Per Share': '$0.25', 'Record Date': 'August 12, 2024', 'Payment Date': 'August 15, 2024'}</t>
+          <t>{'Issuance Date': 'May 10, 2023', 'Total Principal Amount': '$5,250,000,000', 'Issuer': 'Apple Inc.', 'Debt Type': 'Senior Unsecured Notes', '2026 Notes Principal Amount': '$1,000,000,000', '2026 Notes Interest Rate': '4.421%', '2026 Notes Maturity': 'May 8, 2026', '2028 Notes Principal Amount': '$1,500,000,000', '2028 Notes Interest Rate': '4.000%', '2028 Notes Maturity': 'May 10, 2028', '2030 Notes Principal Amount': '$500,000,000', '2030 Notes Interest Rate': '4.150%', '2030 Notes Maturity': 'May 10, 2030', '2033 Notes Principal Amount': '$1,000,000,000', '2033 Notes Interest Rate': '4.300%', '2033 Notes Maturity': 'May 10, 2033', '2053 Notes Principal Amount': '$1,250,000,000', '2053 Notes Interest Rate': '4.850%', '2053 Notes Maturity': 'May 10, 2053', 'Underwriters': 'Goldman Sachs &amp; Co. LLC, Barclays Capital Inc., J.P. Morgan Securities LLC'}</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{'Shareholder Returns': 'Direct return of capital to shareholders', 'Cash Flow Impact': 'Future cash outflow for dividend payment', 'Capital Allocation Strategy': 'Demonstrates an ongoing commitment to shareholder distributions'}</t>
+          <t>{'Leverage': 'Increase', 'Interest Expense': 'Increase', 'Liquidity': 'Increase', 'Debt Structure': 'Diversified maturities with fixed interest rates', 'Cost of Debt': 'Reflects prevailing market rates for long-term corporate debt'}</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.439</v>
+        <v>0.237</v>
       </c>
       <c r="H7" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="I7" t="n">
-        <v>0.22</v>
+        <v>0.166</v>
       </c>
     </row>
   </sheetData>
@@ -1328,7 +1328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>-0.6662322494870978</v>
+        <v>-0.869684734292391</v>
       </c>
     </row>
     <row r="6">
@@ -1411,7 +1411,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1338363006801.892</v>
+        <v>583808687846.8268</v>
       </c>
     </row>
     <row r="9">
@@ -1431,7 +1431,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1237861006801.892</v>
+        <v>483306687846.8268</v>
       </c>
     </row>
     <row r="11">
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1237861006801.892</v>
+        <v>483306687846.8268</v>
       </c>
     </row>
     <row r="12">
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>84.31640913456937</v>
+        <v>32.92024242305617</v>
       </c>
     </row>
     <row r="13">
@@ -1461,7 +1461,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>286092661542.4216</v>
+        <v>125479882016.0124</v>
       </c>
     </row>
     <row r="14">
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1527467145118.812</v>
+        <v>666332116795.1959</v>
       </c>
     </row>
     <row r="15">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.7862368728899202</v>
+        <v>0.7850667785044432</v>
       </c>
     </row>
     <row r="16">
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.07738</v>
+        <v>0.077712</v>
       </c>
     </row>
     <row r="18">
@@ -1596,7 +1596,7 @@
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>0</v>
+        <v>0.000332</v>
       </c>
     </row>
     <row r="28">
@@ -1645,7 +1645,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>78057296645.19353</v>
+        <v>34267022966.34963</v>
       </c>
     </row>
     <row r="34">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>0.07738</v>
+        <v>0.077712</v>
       </c>
     </row>
     <row r="37">
@@ -1685,7 +1685,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>0.008144933451307443</v>
+        <v>0.008476933451307442</v>
       </c>
     </row>
     <row r="38">
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>0.7862368728899202</v>
+        <v>0.7850667785044432</v>
       </c>
     </row>
     <row r="39">
@@ -1733,15 +1733,35 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
           <t>growth</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>margin</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>nopat</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>reinvestment</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
         <is>
           <t>projected_cf</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>discounted_cf</t>
         </is>
@@ -1751,56 +1771,104 @@
       <c r="A44" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="4" t="n">
+      <c r="B44" s="5" t="n">
+        <v>153708956226.7738</v>
+      </c>
+      <c r="C44" s="4" t="n">
         <v>0.06923506654869256</v>
       </c>
-      <c r="C44" s="5" t="n">
-        <v>63613284896.26122</v>
-      </c>
-      <c r="D44" s="5" t="n">
-        <v>59044427125.30511</v>
+      <c r="D44" s="4" t="n">
+        <v>0.2669402661947702</v>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>32414576656.43929</v>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>4488450743.91254</v>
+      </c>
+      <c r="G44" s="5" t="n">
+        <v>27926125912.52674</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>25912419934.57134</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B45" s="4" t="n">
+      <c r="B45" s="5" t="n">
+        <v>164351006040.2646</v>
+      </c>
+      <c r="C45" s="4" t="n">
         <v>0.06923506654869256</v>
       </c>
-      <c r="C45" s="5" t="n">
-        <v>68017554909.43481</v>
-      </c>
-      <c r="D45" s="5" t="n">
-        <v>58598054508.76667</v>
+      <c r="D45" s="4" t="n">
+        <v>0.2669402661947702</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>34658802028.39555</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>4799208929.867854</v>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>29859593098.5277</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>25708601234.0765</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B46" s="4" t="n">
+      <c r="B46" s="5" t="n">
+        <v>175729858880.8069</v>
+      </c>
+      <c r="C46" s="4" t="n">
         <v>0.06923506654869256</v>
       </c>
-      <c r="C46" s="5" t="n">
-        <v>72726754850.06888</v>
-      </c>
-      <c r="D46" s="5" t="n">
-        <v>58155056444.62032</v>
+      <c r="D46" s="4" t="n">
+        <v>0.2669402661947702</v>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>37058406493.32948</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>5131482479.508333</v>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>31926924013.82114</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>25506385705.44967</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B47" s="4" t="n">
+      <c r="B47" s="5" t="n">
+        <v>184009816353.9195</v>
+      </c>
+      <c r="C47" s="4" t="n">
         <v>0.04711753327434628</v>
       </c>
-      <c r="C47" s="5" t="n">
-        <v>76153460141.65222</v>
-      </c>
-      <c r="D47" s="5" t="n">
-        <v>56521542307.93333</v>
+      <c r="D47" s="4" t="n">
+        <v>0.2669402661947702</v>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>38804507194.37318</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>5373265275.983294</v>
+      </c>
+      <c r="G47" s="5" t="n">
+        <v>33431241918.38989</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>24782301470.74034</v>
       </c>
     </row>
     <row r="48">
@@ -1808,13 +1876,25 @@
         <v>5</v>
       </c>
       <c r="B48" t="n">
+        <v>188610061762.7674</v>
+      </c>
+      <c r="C48" t="n">
         <v>0.025</v>
       </c>
-      <c r="C48" t="n">
-        <v>78057296645.19353</v>
-      </c>
       <c r="D48" t="n">
-        <v>53773581155.79616</v>
+        <v>0.2669402661947702</v>
+      </c>
+      <c r="E48" t="n">
+        <v>39774619874.23251</v>
+      </c>
+      <c r="F48" t="n">
+        <v>5507596907.882874</v>
+      </c>
+      <c r="G48" t="n">
+        <v>34267022966.34963</v>
+      </c>
+      <c r="H48" t="n">
+        <v>23570173671.17453</v>
       </c>
     </row>
   </sheetData>
@@ -1865,16 +1945,16 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>869215489659.3091</v>
+        <v>336771374964.6568</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>-0.7656311192448856</v>
+        <v>-0.9091954398422377</v>
       </c>
       <c r="D2" s="6" t="n">
         <v>0.05538805323895405</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>0.09412</v>
+        <v>0.09445199999999999</v>
       </c>
     </row>
     <row r="3">
@@ -1884,16 +1964,16 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>1237861006801.892</v>
+        <v>483306687846.8268</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>-0.6662322494870978</v>
+        <v>-0.869684734292391</v>
       </c>
       <c r="D3" s="6" t="n">
         <v>0.06923506654869256</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>0.07738</v>
+        <v>0.077712</v>
       </c>
     </row>
     <row r="4">
@@ -1903,10 +1983,10 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>831810025739.7334</v>
+        <v>295624937015.8509</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>-0.7757168538150241</v>
+        <v>-0.9202898631743635</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>0.08308207985843107</v>
@@ -1971,22 +2051,22 @@
         <v>0.03</v>
       </c>
       <c r="B2" s="7" t="n">
-        <v>86.96131101218172</v>
+        <v>36.17431844927718</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>69.89140126856249</v>
+        <v>28.34603998629831</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>58.07410742217829</v>
+        <v>22.9266166678521</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>49.40837190210377</v>
+        <v>18.95250129427619</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>42.78187058802786</v>
+        <v>15.91358086054207</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>37.55062675921888</v>
+        <v>13.51452696894406</v>
       </c>
     </row>
     <row r="3">
@@ -1994,22 +2074,22 @@
         <v>0.04</v>
       </c>
       <c r="B3" s="7" t="n">
-        <v>90.01959173501793</v>
+        <v>37.57684918762927</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>72.36457204970058</v>
+        <v>29.4802386933822</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>60.14289634050361</v>
+        <v>23.87536542968014</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>51.18119259875603</v>
+        <v>19.7655187200721</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>44.32885357653025</v>
+        <v>16.62302887716175</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>38.91973946915284</v>
+        <v>14.1424034897659</v>
       </c>
     </row>
     <row r="4">
@@ -2017,22 +2097,22 @@
         <v>0.05</v>
       </c>
       <c r="B4" s="7" t="n">
-        <v>93.15185958279734</v>
+        <v>39.0133104988684</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>74.89710832657362</v>
+        <v>30.64166247890449</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>62.26095835416056</v>
+        <v>24.84671088456531</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>52.99591046496124</v>
+        <v>20.59775023164805</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>45.9121146367611</v>
+        <v>17.34911405542179</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>40.32071243537611</v>
+        <v>14.78489115744679</v>
       </c>
     </row>
     <row r="5">
@@ -2040,22 +2120,22 @@
         <v>0.06</v>
       </c>
       <c r="B5" s="7" t="n">
-        <v>96.35928227418276</v>
+        <v>39.43246253165267</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>77.48994272066746</v>
+        <v>30.97126365028848</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>64.42906397208012</v>
+        <v>25.11463616506244</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>54.85317766387584</v>
+        <v>20.82071383199625</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>47.53221588570802</v>
+        <v>17.5379220081349</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>41.75403707455268</v>
+        <v>14.94692935814776</v>
       </c>
     </row>
     <row r="6">
@@ -2063,22 +2143,22 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="B6" s="7" t="n">
-        <v>66.6479894802048</v>
+        <v>25.36064076441032</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>80.14401487225619</v>
+        <v>31.27485250954388</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>66.6479894802048</v>
+        <v>25.36064076441032</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>56.75365123008976</v>
+        <v>21.02475595467822</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>49.18972362355476</v>
+        <v>17.71010084768234</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>43.22020844684365</v>
+        <v>15.09414720612718</v>
       </c>
     </row>
     <row r="7">
@@ -2086,22 +2166,22 @@
         <v>0.08000000000000002</v>
       </c>
       <c r="B7" s="7" t="n">
-        <v>58.69799306962638</v>
+        <v>21.20883894808658</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>58.69799306962638</v>
+        <v>21.20883894808658</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>68.91851694148886</v>
+        <v>25.58350569018493</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>58.69799306962639</v>
+        <v>21.20883894808658</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>50.88520833368126</v>
+        <v>17.86475111305817</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>44.7197252559071</v>
+        <v>15.22575392392546</v>
       </c>
     </row>
     <row r="8">
@@ -2109,22 +2189,22 @@
         <v>0.09000000000000001</v>
       </c>
       <c r="B8" s="7" t="n">
-        <v>52.61924468266356</v>
+        <v>18.00095183565742</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>52.61924468266356</v>
+        <v>18.00095183565742</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>52.61924468266356</v>
+        <v>18.00095183565742</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>60.68686995994259</v>
+        <v>21.37190021378385</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>52.61924468266363</v>
+        <v>18.00095183565745</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>46.25308984889815</v>
+        <v>15.34093992704519</v>
       </c>
     </row>
     <row r="9">
@@ -2132,22 +2212,22 @@
         <v>0.1</v>
       </c>
       <c r="B9" s="7" t="n">
-        <v>47.82080821646895</v>
+        <v>15.43887663829424</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>47.82080821646895</v>
+        <v>15.43887663829424</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>47.82080821646895</v>
+        <v>15.43887663829424</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>47.82080821646895</v>
+        <v>15.43887663829424</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>54.39241152027419</v>
+        <v>18.11776032611869</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>47.82080821646901</v>
+        <v>15.43887663829426</v>
       </c>
     </row>
   </sheetData>
@@ -2161,268 +2241,311 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>The model estimates an intrinsic value of $84.32, implying -66.6% upside from the current price of $252.62.
-Under a bear case, value falls to $59.21, while the bull case reaches $56.66.
-Growth is driven by an estimated ROIC of 50.0% and reinvestment rate of 10.0%.</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>--- SUMMARY ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>--- SUMMARY ---</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+          <t>Intrinsic Value</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>32.92024242305617</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Investment Signal</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
+          <t>Current Price</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>252.62</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Intrinsic Value (Base Case)</t>
+          <t>Upside (%)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>84.31640913456937</v>
+        <v>-0.869684734292391</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Current Price</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>252.62</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Upside (%)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>-0.6662322494870978</v>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>--- ANALYST VIEW ---</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>We formally initiate coverage with an absolute SELL rating assignment. Our rigorously defined base case DCF natively yields an intrinsic value of $32.92, implying an absolute -87.0% return against observed execution levels of $252.62. Boundary valuation scenarios rigidly restrict the underlying asset constraints between $22.94 (Bear downside) and $20.14 (Assumed Bull execution). Downstream forward growth lines securely modeled against 6.9% limits, rigorously guarded by a native applied discount rate threshold boundary of 7.8%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>--- ANALYST SUMMARY BLOCK ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Rating: SELL
+Reason:
+- Strong baseline revenue growth projected at 6.9%
+- High returns on invested capital (50.0%), implying efficient scalable reinvestment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>--- SCENARIOS ---</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Bear Value</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>59.206266656357</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Base Value</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>84.31640913456937</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Bull Value</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>56.65840838924861</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>--- DRIVERS ---</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+          <t>Bear Value</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>22.93904798705392</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Growth Assumption (Stage 1)</t>
+          <t>Base Value</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>0.06923506654869256</v>
+        <v>32.92024242305617</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Discount Rate</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>0.07738</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>ROIC</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>0.5</v>
+          <t>Bull Value</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>20.1363747648923</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Reinvestment Rate</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>0.1</v>
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>--- DRIVERS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>--- RISK SUMMARY ---</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Driver 1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Strong baseline revenue growth projected at 6.9%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Driver 2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>High returns on invested capital (50.0%), implying efficient scalable reinvestment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>--- RISKS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Key Risks</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>A U.S. District Court granted preliminary approval for the proposed settlement of consolidated shareholder derivative lawsuits against Apple Inc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Risk Score</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>24</v>
-      </c>
-    </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>--- VALUATION DIAGNOSTICS ---</t>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Risk 2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Event Risk Threat: Apple Inc. amended and restated its Non-Employee Director Stock Plan, effective February 24, 2026, establishing an aggregate limit of 44.8 million shares for awards and an annual compensation cap of $1.5 million per non-employee director.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Risk 3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Event Risk Threat: A U.S. District Court granted preliminary approval for the proposed settlement of consolidated shareholder derivative lawsuits against Apple Inc. on April 23, 2024.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Risk 4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Event Risk Threat: Apple Inc. consummated the issuance and sale of $5.25 billion in aggregate principal amount across five series of senior unsecured notes with varying interest rates and maturities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>--- DIAGNOSTICS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Terminal Value Contribution (%)</t>
         </is>
       </c>
-      <c r="B30" s="4" t="n">
-        <v>0.7862368728899202</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="B34" s="4" t="n">
+        <v>0.7850667785044432</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Spread (Discount - Growth)</t>
         </is>
       </c>
-      <c r="B31" t="n">
-        <v>0.008144933451307443</v>
+      <c r="B35" s="4" t="n">
+        <v>0.008476933451307442</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Overall Operational Risk Score</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>